<commit_message>
Optimize requisition change workflow: remove dismissal logic, rename sections to 'Demand Change Alert', and add persistent change flow history.
</commit_message>
<xml_diff>
--- a/Newdata/今日入庫.xlsx
+++ b/Newdata/今日入庫.xlsx
@@ -11,32 +11,50 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="59">
+  <si>
+    <t>1600001665</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>PCMCIA CABLE (委託FANUC處理)</t>
+  </si>
+  <si>
+    <t>4T0010</t>
+  </si>
+  <si>
+    <t>101</t>
+  </si>
+  <si>
+    <t>陳彥融取</t>
+  </si>
+  <si>
+    <t>5000023180</t>
+  </si>
+  <si>
+    <t>EA</t>
+  </si>
+  <si>
+    <t>2000007630</t>
+  </si>
   <si>
     <t>1400093971</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>一廠封箱上車</t>
   </si>
   <si>
     <t>2L0003</t>
   </si>
   <si>
-    <t>101</t>
-  </si>
-  <si>
     <t>5000022887</t>
   </si>
   <si>
-    <t>EA</t>
-  </si>
-  <si>
     <t>100003502</t>
   </si>
   <si>
@@ -74,6 +92,60 @@
   </si>
   <si>
     <t>5000022888</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>8315000470A1</t>
+  </si>
+  <si>
+    <t>Z軸上斜楔_280*239*40(1.5/100)</t>
+  </si>
+  <si>
+    <t>0105</t>
+  </si>
+  <si>
+    <t>3926042199</t>
+  </si>
+  <si>
+    <t>5000023185</t>
+  </si>
+  <si>
+    <t>400006372</t>
+  </si>
+  <si>
+    <t>8810001317A3</t>
+  </si>
+  <si>
+    <t>底座加工圖_5970*2230*558,HSA-327</t>
+  </si>
+  <si>
+    <t>06</t>
+  </si>
+  <si>
+    <t>008529</t>
+  </si>
+  <si>
+    <t>5000023183</t>
+  </si>
+  <si>
+    <t>400006466</t>
+  </si>
+  <si>
+    <t>8813001120B3</t>
+  </si>
+  <si>
+    <t>工作台加工圖_HSA-323/327,3000x2200mm</t>
+  </si>
+  <si>
+    <t>008528</t>
+  </si>
+  <si>
+    <t>5000023184</t>
+  </si>
+  <si>
+    <t>400005799</t>
   </si>
   <si>
     <t>採購單</t>
@@ -226,7 +298,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="12" customWidth="1"/>
@@ -236,7 +308,7 @@
     <col min="5" max="5" bestFit="1" width="8" customWidth="1"/>
     <col min="6" max="6" bestFit="1" width="6" customWidth="1"/>
     <col min="7" max="7" bestFit="1" width="6" customWidth="1"/>
-    <col min="8" max="8" bestFit="1" width="8" customWidth="1"/>
+    <col min="8" max="8" bestFit="1" width="12" customWidth="1"/>
     <col min="9" max="9" bestFit="1" width="12" customWidth="1"/>
     <col min="10" max="10" bestFit="1" width="13" customWidth="1"/>
     <col min="11" max="11" bestFit="1" width="13" customWidth="1"/>
@@ -247,46 +319,46 @@
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -312,10 +384,10 @@
         <v>5</v>
       </c>
       <c r="H2" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J2" s="2">
         <v>46141</v>
@@ -327,15 +399,15 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:14">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
@@ -344,10 +416,10 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F3" t="s">
         <v>2</v>
@@ -356,7 +428,7 @@
         <v>5</v>
       </c>
       <c r="H3" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="I3" t="s">
         <v>13</v>
@@ -371,7 +443,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N3" t="s">
         <v>14</v>
@@ -385,79 +457,255 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
         <v>16</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>17</v>
       </c>
-      <c r="E4" t="s">
-        <v>18</v>
-      </c>
       <c r="F4" t="s">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="G4" t="s">
         <v>5</v>
       </c>
       <c r="H4" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="I4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="2">
+        <v>46141</v>
+      </c>
+      <c r="K4" s="2">
+        <v>46141</v>
+      </c>
+      <c r="L4" s="3">
+        <v>1</v>
+      </c>
+      <c r="M4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N4" t="s">
         <v>20</v>
       </c>
-      <c r="J4" s="2">
-        <v>46141</v>
-      </c>
-      <c r="K4" s="2">
-        <v>46141</v>
-      </c>
-      <c r="L4" s="3">
-        <v>2</v>
-      </c>
-      <c r="M4" t="s">
-        <v>7</v>
-      </c>
-      <c r="N4" t="s">
-        <v>2</v>
-      </c>
     </row>
     <row r="5" spans="1:14">
-      <c r="A5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="6">
-        <v>4</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="N5" s="4" t="s">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H5" t="s">
+        <v>2</v>
+      </c>
+      <c r="I5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" s="2">
+        <v>46141</v>
+      </c>
+      <c r="K5" s="2">
+        <v>46141</v>
+      </c>
+      <c r="L5" s="3">
+        <v>2</v>
+      </c>
+      <c r="M5" t="s">
+        <v>8</v>
+      </c>
+      <c r="N5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" t="s">
+        <v>5</v>
+      </c>
+      <c r="H6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J6" s="2">
+        <v>46141</v>
+      </c>
+      <c r="K6" s="2">
+        <v>46141</v>
+      </c>
+      <c r="L6" s="3">
+        <v>40</v>
+      </c>
+      <c r="M6" t="s">
+        <v>8</v>
+      </c>
+      <c r="N6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" t="s">
+        <v>2</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" t="s">
+        <v>5</v>
+      </c>
+      <c r="H7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" s="2">
+        <v>46141</v>
+      </c>
+      <c r="K7" s="2">
+        <v>46141</v>
+      </c>
+      <c r="L7" s="3">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
+        <v>8</v>
+      </c>
+      <c r="N7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" t="s">
+        <v>2</v>
+      </c>
+      <c r="F8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G8" t="s">
+        <v>5</v>
+      </c>
+      <c r="H8" t="s">
+        <v>42</v>
+      </c>
+      <c r="I8" t="s">
+        <v>43</v>
+      </c>
+      <c r="J8" s="2">
+        <v>46141</v>
+      </c>
+      <c r="K8" s="2">
+        <v>46141</v>
+      </c>
+      <c r="L8" s="3">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
+        <v>8</v>
+      </c>
+      <c r="N8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="6">
+        <v>47</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N9" s="4" t="s">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix requisition alert log being overwritten by status updates.
</commit_message>
<xml_diff>
--- a/Newdata/今日入庫.xlsx
+++ b/Newdata/今日入庫.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="68">
   <si>
     <t>1600001665</t>
   </si>
@@ -92,6 +92,33 @@
   </si>
   <si>
     <t>5000022888</t>
+  </si>
+  <si>
+    <t>1100097760</t>
+  </si>
+  <si>
+    <t>772700010700</t>
+  </si>
+  <si>
+    <t>H-plus 3-SSD(SATA)_SQF-S25M8-64G-SAC</t>
+  </si>
+  <si>
+    <t>4E0008</t>
+  </si>
+  <si>
+    <t>09</t>
+  </si>
+  <si>
+    <t>售服MRP</t>
+  </si>
+  <si>
+    <t>5000023191</t>
+  </si>
+  <si>
+    <t>1100097275</t>
+  </si>
+  <si>
+    <t>5000023192</t>
   </si>
   <si>
     <t>0</t>
@@ -298,13 +325,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="12" customWidth="1"/>
     <col min="2" max="2" bestFit="1" width="4" customWidth="1"/>
     <col min="3" max="3" bestFit="1" width="14" customWidth="1"/>
-    <col min="4" max="4" bestFit="1" width="37" customWidth="1"/>
+    <col min="4" max="4" bestFit="1" width="38" customWidth="1"/>
     <col min="5" max="5" bestFit="1" width="8" customWidth="1"/>
     <col min="6" max="6" bestFit="1" width="6" customWidth="1"/>
     <col min="7" max="7" bestFit="1" width="6" customWidth="1"/>
@@ -319,46 +346,46 @@
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -539,10 +566,10 @@
     </row>
     <row r="6" spans="1:14">
       <c r="A6" t="s">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="C6" t="s">
         <v>28</v>
@@ -551,19 +578,19 @@
         <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G6" t="s">
         <v>5</v>
       </c>
       <c r="H6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J6" s="2">
         <v>46141</v>
@@ -572,42 +599,42 @@
         <v>46141</v>
       </c>
       <c r="L6" s="3">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="M6" t="s">
         <v>8</v>
       </c>
       <c r="N6" t="s">
-        <v>33</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" t="s">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D7" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E7" t="s">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="F7" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G7" t="s">
         <v>5</v>
       </c>
       <c r="H7" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="I7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J7" s="2">
         <v>46141</v>
@@ -622,7 +649,7 @@
         <v>8</v>
       </c>
       <c r="N7" t="s">
-        <v>39</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -630,82 +657,170 @@
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E8" t="s">
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G8" t="s">
         <v>5</v>
       </c>
       <c r="H8" t="s">
+        <v>40</v>
+      </c>
+      <c r="I8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J8" s="2">
+        <v>46141</v>
+      </c>
+      <c r="K8" s="2">
+        <v>46141</v>
+      </c>
+      <c r="L8" s="3">
+        <v>40</v>
+      </c>
+      <c r="M8" t="s">
+        <v>8</v>
+      </c>
+      <c r="N8" t="s">
         <v>42</v>
       </c>
-      <c r="I8" t="s">
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
         <v>43</v>
       </c>
-      <c r="J8" s="2">
-        <v>46141</v>
-      </c>
-      <c r="K8" s="2">
-        <v>46141</v>
-      </c>
-      <c r="L8" s="3">
-        <v>1</v>
-      </c>
-      <c r="M8" t="s">
-        <v>8</v>
-      </c>
-      <c r="N8" t="s">
+      <c r="D9" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="9" spans="1:14">
-      <c r="A9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="6">
+      <c r="E9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F9" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" t="s">
+        <v>5</v>
+      </c>
+      <c r="H9" t="s">
+        <v>46</v>
+      </c>
+      <c r="I9" t="s">
         <v>47</v>
       </c>
-      <c r="M9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N9" s="4" t="s">
+      <c r="J9" s="2">
+        <v>46141</v>
+      </c>
+      <c r="K9" s="2">
+        <v>46141</v>
+      </c>
+      <c r="L9" s="3">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
+        <v>8</v>
+      </c>
+      <c r="N9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F10" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H10" t="s">
+        <v>51</v>
+      </c>
+      <c r="I10" t="s">
+        <v>52</v>
+      </c>
+      <c r="J10" s="2">
+        <v>46141</v>
+      </c>
+      <c r="K10" s="2">
+        <v>46141</v>
+      </c>
+      <c r="L10" s="3">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
+        <v>8</v>
+      </c>
+      <c r="N10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="6">
+        <v>49</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N11" s="4" t="s">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data and fix requisition logging
</commit_message>
<xml_diff>
--- a/Newdata/今日入庫.xlsx
+++ b/Newdata/今日入庫.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="74">
   <si>
     <t>1600001665</t>
   </si>
@@ -119,6 +119,24 @@
   </si>
   <si>
     <t>5000023192</t>
+  </si>
+  <si>
+    <t>1100094374</t>
+  </si>
+  <si>
+    <t>8015003001C0</t>
+  </si>
+  <si>
+    <t>接頭座,EM耦合接頭用,AC獨立_L418.5*W428*H86</t>
+  </si>
+  <si>
+    <t>1G0052</t>
+  </si>
+  <si>
+    <t>0101</t>
+  </si>
+  <si>
+    <t>5000023193</t>
   </si>
   <si>
     <t>0</t>
@@ -325,7 +343,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="12" customWidth="1"/>
@@ -346,46 +364,46 @@
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -654,10 +672,10 @@
     </row>
     <row r="8" spans="1:14">
       <c r="A8" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
@@ -666,16 +684,16 @@
         <v>38</v>
       </c>
       <c r="E8" t="s">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="F8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G8" t="s">
         <v>5</v>
       </c>
       <c r="H8" t="s">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="I8" t="s">
         <v>41</v>
@@ -687,13 +705,13 @@
         <v>46141</v>
       </c>
       <c r="L8" s="3">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="M8" t="s">
         <v>8</v>
       </c>
       <c r="N8" t="s">
-        <v>42</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -701,7 +719,7 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
         <v>43</v>
@@ -731,7 +749,7 @@
         <v>46141</v>
       </c>
       <c r="L9" s="3">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="M9" t="s">
         <v>8</v>
@@ -745,7 +763,7 @@
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
         <v>49</v>
@@ -757,70 +775,114 @@
         <v>2</v>
       </c>
       <c r="F10" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="G10" t="s">
         <v>5</v>
       </c>
       <c r="H10" t="s">
+        <v>52</v>
+      </c>
+      <c r="I10" t="s">
+        <v>53</v>
+      </c>
+      <c r="J10" s="2">
+        <v>46141</v>
+      </c>
+      <c r="K10" s="2">
+        <v>46141</v>
+      </c>
+      <c r="L10" s="3">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
+        <v>8</v>
+      </c>
+      <c r="N10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" t="s">
+        <v>2</v>
+      </c>
+      <c r="F11" t="s">
         <v>51</v>
       </c>
-      <c r="I10" t="s">
+      <c r="G11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H11" t="s">
+        <v>57</v>
+      </c>
+      <c r="I11" t="s">
+        <v>58</v>
+      </c>
+      <c r="J11" s="2">
+        <v>46141</v>
+      </c>
+      <c r="K11" s="2">
+        <v>46141</v>
+      </c>
+      <c r="L11" s="3">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
+        <v>8</v>
+      </c>
+      <c r="N11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="6">
         <v>52</v>
       </c>
-      <c r="J10" s="2">
-        <v>46141</v>
-      </c>
-      <c r="K10" s="2">
-        <v>46141</v>
-      </c>
-      <c r="L10" s="3">
-        <v>1</v>
-      </c>
-      <c r="M10" t="s">
-        <v>8</v>
-      </c>
-      <c r="N10" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
-      <c r="A11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="6">
-        <v>49</v>
-      </c>
-      <c r="M11" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N11" s="4" t="s">
+      <c r="M12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N12" s="4" t="s">
         <v>2</v>
       </c>
     </row>

</xml_diff>